<commit_message>
Added Working prototype of Data Driven Testing
</commit_message>
<xml_diff>
--- a/Test_Data/Compound.xlsx
+++ b/Test_Data/Compound.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="9">
   <si>
     <t>Principle</t>
   </si>
@@ -54,6 +54,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -61,7 +62,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -72,6 +73,26 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="17"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,11 +123,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -258,71 +287,71 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="0">
         <v>1000</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="0">
         <v>5</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="0">
         <v>2</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="0">
         <v>1100</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="0">
+        <v>50000</v>
+      </c>
+      <c r="B3" s="0">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0">
+        <v>10</v>
+      </c>
+      <c r="D3" s="0">
+        <v>60000</v>
+      </c>
+      <c r="E3" t="s" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="0">
+        <v>25000</v>
+      </c>
+      <c r="B4" s="0">
+        <v>1</v>
+      </c>
+      <c r="C4" s="0">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s" s="8">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>50000</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-      <c r="D3">
-        <v>60000</v>
-      </c>
-      <c r="E3" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="0">
+        <v>5025</v>
+      </c>
+      <c r="B5" s="0">
+        <v>0</v>
+      </c>
+      <c r="C5" s="0">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s" s="9">
         <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>25000</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>5025</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>